<commit_message>
feat: wire Monte Carlo simulation + portfolio selection into dashboard (generate pool → simulate → select best)
</commit_message>
<xml_diff>
--- a/data/live/BallparkPal_Games_2026-04-12.xlsx
+++ b/data/live/BallparkPal_Games_2026-04-12.xlsx
@@ -638,109 +638,109 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>4.738</v>
+        <v>4.793</v>
       </c>
       <c r="F2" t="n">
-        <v>4.127</v>
+        <v>4.147</v>
       </c>
       <c r="G2" t="n">
-        <v>0.532</v>
+        <v>0.541</v>
       </c>
       <c r="H2" t="n">
-        <v>0.468</v>
+        <v>0.459</v>
       </c>
       <c r="I2" t="n">
-        <v>0.3</v>
+        <v>0.303</v>
       </c>
       <c r="J2" t="n">
-        <v>0.101</v>
+        <v>0.104</v>
       </c>
       <c r="K2" t="n">
-        <v>0.131</v>
+        <v>0.135</v>
       </c>
       <c r="L2" t="n">
         <v>0.188</v>
       </c>
       <c r="M2" t="n">
-        <v>0.099</v>
+        <v>0.096</v>
       </c>
       <c r="N2" t="n">
-        <v>0.181</v>
+        <v>0.175</v>
       </c>
       <c r="O2" t="n">
-        <v>0.509</v>
+        <v>0.502</v>
       </c>
       <c r="P2" t="n">
-        <v>2.895</v>
+        <v>2.884</v>
       </c>
       <c r="Q2" t="n">
-        <v>2.241</v>
+        <v>2.277</v>
       </c>
       <c r="R2" t="n">
         <v>0.507</v>
       </c>
       <c r="S2" t="n">
-        <v>0.34</v>
+        <v>0.344</v>
       </c>
       <c r="T2" t="n">
         <v>0</v>
       </c>
       <c r="U2" t="n">
-        <v>0.011</v>
+        <v>0.013</v>
       </c>
       <c r="V2" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="W2" t="n">
-        <v>0.054</v>
+        <v>0.05</v>
       </c>
       <c r="X2" t="n">
         <v>0.039</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.105</v>
+        <v>0.096</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.075</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.123</v>
+        <v>0.124</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.079</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.118</v>
+        <v>0.108</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.066</v>
+        <v>0.065</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.082</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="AF2" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="AG2" t="n">
         <v>0.052</v>
       </c>
-      <c r="AG2" t="n">
-        <v>0.053</v>
-      </c>
       <c r="AH2" t="n">
-        <v>0.04</v>
+        <v>0.035</v>
       </c>
       <c r="AI2" t="n">
         <v>0.031</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0.016</v>
+        <v>0.021</v>
       </c>
       <c r="AK2" t="n">
-        <v>0.02</v>
+        <v>0.014</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.006</v>
+        <v>0.01</v>
       </c>
       <c r="AM2" t="n">
-        <v>0.006</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="AN2" t="n">
         <v>0.014</v>
@@ -766,112 +766,112 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>3.934</v>
+        <v>3.941</v>
       </c>
       <c r="F3" t="n">
-        <v>4.365</v>
+        <v>4.426</v>
       </c>
       <c r="G3" t="n">
-        <v>0.43</v>
+        <v>0.426</v>
       </c>
       <c r="H3" t="n">
-        <v>0.57</v>
+        <v>0.574</v>
       </c>
       <c r="I3" t="n">
-        <v>0.212</v>
+        <v>0.21</v>
       </c>
       <c r="J3" t="n">
-        <v>0.094</v>
+        <v>0.089</v>
       </c>
       <c r="K3" t="n">
-        <v>0.124</v>
+        <v>0.127</v>
       </c>
       <c r="L3" t="n">
-        <v>0.275</v>
+        <v>0.279</v>
       </c>
       <c r="M3" t="n">
-        <v>0.108</v>
+        <v>0.11</v>
       </c>
       <c r="N3" t="n">
-        <v>0.187</v>
+        <v>0.186</v>
       </c>
       <c r="O3" t="n">
-        <v>0.463</v>
+        <v>0.471</v>
       </c>
       <c r="P3" t="n">
-        <v>2.066</v>
+        <v>2.023</v>
       </c>
       <c r="Q3" t="n">
-        <v>2.488</v>
+        <v>2.513</v>
       </c>
       <c r="R3" t="n">
-        <v>0.364</v>
+        <v>0.353</v>
       </c>
       <c r="S3" t="n">
-        <v>0.466</v>
+        <v>0.482</v>
       </c>
       <c r="T3" t="n">
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>0.02</v>
+        <v>0.023</v>
       </c>
       <c r="V3" t="n">
-        <v>0.026</v>
+        <v>0.017</v>
       </c>
       <c r="W3" t="n">
-        <v>0.075</v>
+        <v>0.065</v>
       </c>
       <c r="X3" t="n">
-        <v>0.054</v>
+        <v>0.056</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.105</v>
+        <v>0.107</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.077</v>
+        <v>0.079</v>
       </c>
       <c r="AA3" t="n">
         <v>0.117</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.08</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.103</v>
+        <v>0.109</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.065</v>
+        <v>0.062</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.079</v>
       </c>
       <c r="AF3" t="n">
-        <v>0.044</v>
+        <v>0.042</v>
       </c>
       <c r="AG3" t="n">
-        <v>0.054</v>
+        <v>0.05</v>
       </c>
       <c r="AH3" t="n">
-        <v>0.028</v>
+        <v>0.027</v>
       </c>
       <c r="AI3" t="n">
-        <v>0.029</v>
+        <v>0.024</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0.015</v>
+        <v>0.017</v>
       </c>
       <c r="AK3" t="n">
-        <v>0.015</v>
+        <v>0.014</v>
       </c>
       <c r="AL3" t="n">
-        <v>0.006</v>
+        <v>0.007</v>
       </c>
       <c r="AM3" t="n">
-        <v>0.005</v>
+        <v>0.008</v>
       </c>
       <c r="AN3" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="4">
@@ -894,112 +894,112 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>4.42</v>
+        <v>4.257</v>
       </c>
       <c r="F4" t="n">
-        <v>4.775</v>
+        <v>4.543</v>
       </c>
       <c r="G4" t="n">
-        <v>0.433</v>
+        <v>0.436</v>
       </c>
       <c r="H4" t="n">
-        <v>0.5669999999999999</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="I4" t="n">
-        <v>0.228</v>
+        <v>0.25</v>
       </c>
       <c r="J4" t="n">
-        <v>0.089</v>
+        <v>0.079</v>
       </c>
       <c r="K4" t="n">
-        <v>0.116</v>
+        <v>0.106</v>
       </c>
       <c r="L4" t="n">
-        <v>0.271</v>
+        <v>0.267</v>
       </c>
       <c r="M4" t="n">
-        <v>0.111</v>
+        <v>0.113</v>
       </c>
       <c r="N4" t="n">
         <v>0.184</v>
       </c>
       <c r="O4" t="n">
-        <v>0.517</v>
+        <v>0.481</v>
       </c>
       <c r="P4" t="n">
-        <v>2.354</v>
+        <v>2.339</v>
       </c>
       <c r="Q4" t="n">
-        <v>2.654</v>
+        <v>2.536</v>
       </c>
       <c r="R4" t="n">
-        <v>0.389</v>
+        <v>0.401</v>
       </c>
       <c r="S4" t="n">
-        <v>0.466</v>
+        <v>0.452</v>
       </c>
       <c r="T4" t="n">
         <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>0.014</v>
+        <v>0.015</v>
       </c>
       <c r="V4" t="n">
-        <v>0.015</v>
+        <v>0.019</v>
       </c>
       <c r="W4" t="n">
-        <v>0.051</v>
+        <v>0.064</v>
       </c>
       <c r="X4" t="n">
-        <v>0.047</v>
+        <v>0.053</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.092</v>
+        <v>0.1</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.077</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.112</v>
+        <v>0.109</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.081</v>
+        <v>0.08</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.09</v>
+        <v>0.105</v>
       </c>
       <c r="AD4" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="AE4" t="n">
-        <v>0.082</v>
+        <v>0.075</v>
       </c>
       <c r="AF4" t="n">
-        <v>0.05</v>
+        <v>0.053</v>
       </c>
       <c r="AG4" t="n">
-        <v>0.062</v>
+        <v>0.049</v>
       </c>
       <c r="AH4" t="n">
-        <v>0.035</v>
+        <v>0.031</v>
       </c>
       <c r="AI4" t="n">
-        <v>0.036</v>
+        <v>0.031</v>
       </c>
       <c r="AJ4" t="n">
-        <v>0.02</v>
+        <v>0.021</v>
       </c>
       <c r="AK4" t="n">
-        <v>0.022</v>
+        <v>0.018</v>
       </c>
       <c r="AL4" t="n">
         <v>0.01</v>
       </c>
       <c r="AM4" t="n">
-        <v>0.014</v>
+        <v>0.006</v>
       </c>
       <c r="AN4" t="n">
-        <v>0.021</v>
+        <v>0.019</v>
       </c>
     </row>
     <row r="5">
@@ -1022,112 +1022,112 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>3.704</v>
+        <v>3.665</v>
       </c>
       <c r="F5" t="n">
-        <v>4.785</v>
+        <v>4.711</v>
       </c>
       <c r="G5" t="n">
-        <v>0.358</v>
+        <v>0.353</v>
       </c>
       <c r="H5" t="n">
-        <v>0.642</v>
+        <v>0.647</v>
       </c>
       <c r="I5" t="n">
-        <v>0.175</v>
+        <v>0.187</v>
       </c>
       <c r="J5" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.065</v>
       </c>
       <c r="K5" t="n">
-        <v>0.113</v>
+        <v>0.101</v>
       </c>
       <c r="L5" t="n">
-        <v>0.332</v>
+        <v>0.339</v>
       </c>
       <c r="M5" t="n">
-        <v>0.119</v>
+        <v>0.12</v>
       </c>
       <c r="N5" t="n">
-        <v>0.191</v>
+        <v>0.189</v>
       </c>
       <c r="O5" t="n">
-        <v>0.498</v>
+        <v>0.468</v>
       </c>
       <c r="P5" t="n">
-        <v>1.904</v>
+        <v>1.918</v>
       </c>
       <c r="Q5" t="n">
-        <v>2.651</v>
+        <v>2.551</v>
       </c>
       <c r="R5" t="n">
-        <v>0.329</v>
+        <v>0.333</v>
       </c>
       <c r="S5" t="n">
-        <v>0.507</v>
+        <v>0.496</v>
       </c>
       <c r="T5" t="n">
         <v>0</v>
       </c>
       <c r="U5" t="n">
-        <v>0.019</v>
+        <v>0.016</v>
       </c>
       <c r="V5" t="n">
-        <v>0.02</v>
+        <v>0.024</v>
       </c>
       <c r="W5" t="n">
-        <v>0.068</v>
+        <v>0.063</v>
       </c>
       <c r="X5" t="n">
-        <v>0.05</v>
+        <v>0.053</v>
       </c>
       <c r="Y5" t="n">
+        <v>0.107</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>0.129</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>0.08400000000000001</v>
+      </c>
+      <c r="AC5" t="n">
         <v>0.106</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>0.081</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>0.121</v>
-      </c>
-      <c r="AB5" t="n">
-        <v>0.081</v>
-      </c>
-      <c r="AC5" t="n">
-        <v>0.103</v>
       </c>
       <c r="AD5" t="n">
         <v>0.067</v>
       </c>
       <c r="AE5" t="n">
-        <v>0.074</v>
+        <v>0.077</v>
       </c>
       <c r="AF5" t="n">
-        <v>0.046</v>
+        <v>0.043</v>
       </c>
       <c r="AG5" t="n">
         <v>0.049</v>
       </c>
       <c r="AH5" t="n">
-        <v>0.029</v>
+        <v>0.022</v>
       </c>
       <c r="AI5" t="n">
-        <v>0.023</v>
+        <v>0.026</v>
       </c>
       <c r="AJ5" t="n">
-        <v>0.017</v>
+        <v>0.013</v>
       </c>
       <c r="AK5" t="n">
-        <v>0.012</v>
+        <v>0.014</v>
       </c>
       <c r="AL5" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="AM5" t="n">
-        <v>0.008</v>
+        <v>0.007</v>
       </c>
       <c r="AN5" t="n">
-        <v>0.017</v>
+        <v>0.015</v>
       </c>
     </row>
     <row r="6">
@@ -1150,112 +1150,112 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>4.516</v>
+        <v>4.783</v>
       </c>
       <c r="F6" t="n">
-        <v>3.582</v>
+        <v>3.687</v>
       </c>
       <c r="G6" t="n">
-        <v>0.572</v>
+        <v>0.579</v>
       </c>
       <c r="H6" t="n">
-        <v>0.428</v>
+        <v>0.421</v>
       </c>
       <c r="I6" t="n">
-        <v>0.326</v>
+        <v>0.33</v>
       </c>
       <c r="J6" t="n">
-        <v>0.11</v>
+        <v>0.118</v>
       </c>
       <c r="K6" t="n">
-        <v>0.136</v>
+        <v>0.131</v>
       </c>
       <c r="L6" t="n">
-        <v>0.164</v>
+        <v>0.158</v>
       </c>
       <c r="M6" t="n">
         <v>0.081</v>
       </c>
       <c r="N6" t="n">
-        <v>0.183</v>
+        <v>0.182</v>
       </c>
       <c r="O6" t="n">
-        <v>0.519</v>
+        <v>0.498</v>
       </c>
       <c r="P6" t="n">
-        <v>2.712</v>
+        <v>2.799</v>
       </c>
       <c r="Q6" t="n">
-        <v>1.817</v>
+        <v>1.852</v>
       </c>
       <c r="R6" t="n">
-        <v>0.536</v>
+        <v>0.541</v>
       </c>
       <c r="S6" t="n">
-        <v>0.308</v>
+        <v>0.293</v>
       </c>
       <c r="T6" t="n">
         <v>0</v>
       </c>
       <c r="U6" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="V6" t="n">
         <v>0.019</v>
       </c>
-      <c r="V6" t="n">
-        <v>0.018</v>
-      </c>
       <c r="W6" t="n">
-        <v>0.073</v>
+        <v>0.067</v>
       </c>
       <c r="X6" t="n">
-        <v>0.064</v>
+        <v>0.055</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.115</v>
+        <v>0.102</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.129</v>
+        <v>0.127</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.08</v>
+        <v>0.077</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.097</v>
+        <v>0.109</v>
       </c>
       <c r="AD6" t="n">
-        <v>0.066</v>
+        <v>0.061</v>
       </c>
       <c r="AE6" t="n">
-        <v>0.073</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="AF6" t="n">
-        <v>0.041</v>
+        <v>0.048</v>
       </c>
       <c r="AG6" t="n">
-        <v>0.051</v>
+        <v>0.053</v>
       </c>
       <c r="AH6" t="n">
-        <v>0.022</v>
+        <v>0.03</v>
       </c>
       <c r="AI6" t="n">
-        <v>0.024</v>
+        <v>0.03</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0.011</v>
+        <v>0.015</v>
       </c>
       <c r="AK6" t="n">
-        <v>0.015</v>
+        <v>0.013</v>
       </c>
       <c r="AL6" t="n">
-        <v>0.008</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="AM6" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
       <c r="AN6" t="n">
-        <v>0.007</v>
+        <v>0.012</v>
       </c>
     </row>
     <row r="7">
@@ -1278,112 +1278,112 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>3.971</v>
+        <v>3.95</v>
       </c>
       <c r="F7" t="n">
-        <v>4.247</v>
+        <v>4.212</v>
       </c>
       <c r="G7" t="n">
-        <v>0.457</v>
+        <v>0.456</v>
       </c>
       <c r="H7" t="n">
-        <v>0.543</v>
+        <v>0.544</v>
       </c>
       <c r="I7" t="n">
-        <v>0.23</v>
+        <v>0.22</v>
       </c>
       <c r="J7" t="n">
-        <v>0.094</v>
+        <v>0.098</v>
       </c>
       <c r="K7" t="n">
-        <v>0.133</v>
+        <v>0.138</v>
       </c>
       <c r="L7" t="n">
-        <v>0.256</v>
+        <v>0.242</v>
       </c>
       <c r="M7" t="n">
-        <v>0.106</v>
+        <v>0.099</v>
       </c>
       <c r="N7" t="n">
-        <v>0.181</v>
+        <v>0.203</v>
       </c>
       <c r="O7" t="n">
+        <v>0.447</v>
+      </c>
+      <c r="P7" t="n">
+        <v>2.002</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>2.257</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0.385</v>
+      </c>
+      <c r="S7" t="n">
         <v>0.445</v>
-      </c>
-      <c r="P7" t="n">
-        <v>2.096</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>2.264</v>
-      </c>
-      <c r="R7" t="n">
-        <v>0.395</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0.431</v>
       </c>
       <c r="T7" t="n">
         <v>0</v>
       </c>
       <c r="U7" t="n">
-        <v>0.026</v>
+        <v>0.019</v>
       </c>
       <c r="V7" t="n">
-        <v>0.023</v>
+        <v>0.028</v>
       </c>
       <c r="W7" t="n">
-        <v>0.068</v>
+        <v>0.078</v>
       </c>
       <c r="X7" t="n">
-        <v>0.056</v>
+        <v>0.062</v>
       </c>
       <c r="Y7" t="n">
         <v>0.119</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.082</v>
+        <v>0.075</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.119</v>
+        <v>0.127</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.078</v>
+        <v>0.064</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.1</v>
+        <v>0.105</v>
       </c>
       <c r="AD7" t="n">
-        <v>0.062</v>
+        <v>0.063</v>
       </c>
       <c r="AE7" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.067</v>
       </c>
       <c r="AF7" t="n">
-        <v>0.041</v>
+        <v>0.037</v>
       </c>
       <c r="AG7" t="n">
-        <v>0.045</v>
+        <v>0.043</v>
       </c>
       <c r="AH7" t="n">
-        <v>0.026</v>
+        <v>0.025</v>
       </c>
       <c r="AI7" t="n">
-        <v>0.027</v>
+        <v>0.028</v>
       </c>
       <c r="AJ7" t="n">
-        <v>0.016</v>
+        <v>0.018</v>
       </c>
       <c r="AK7" t="n">
-        <v>0.015</v>
+        <v>0.02</v>
       </c>
       <c r="AL7" t="n">
-        <v>0.007</v>
+        <v>0.008</v>
       </c>
       <c r="AM7" t="n">
-        <v>0.007</v>
+        <v>0.005</v>
       </c>
       <c r="AN7" t="n">
-        <v>0.012</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="8">
@@ -1406,16 +1406,16 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>4.28</v>
+        <v>4.294</v>
       </c>
       <c r="F8" t="n">
-        <v>4.233</v>
+        <v>4.276</v>
       </c>
       <c r="G8" t="n">
-        <v>0.474</v>
+        <v>0.481</v>
       </c>
       <c r="H8" t="n">
-        <v>0.526</v>
+        <v>0.519</v>
       </c>
       <c r="I8" t="n">
         <v>0.255</v>
@@ -1424,94 +1424,94 @@
         <v>0.097</v>
       </c>
       <c r="K8" t="n">
-        <v>0.122</v>
+        <v>0.129</v>
       </c>
       <c r="L8" t="n">
-        <v>0.237</v>
+        <v>0.245</v>
       </c>
       <c r="M8" t="n">
-        <v>0.102</v>
+        <v>0.1</v>
       </c>
       <c r="N8" t="n">
-        <v>0.187</v>
+        <v>0.174</v>
       </c>
       <c r="O8" t="n">
-        <v>0.483</v>
+        <v>0.494</v>
       </c>
       <c r="P8" t="n">
-        <v>2.473</v>
+        <v>2.449</v>
       </c>
       <c r="Q8" t="n">
-        <v>2.381</v>
+        <v>2.38</v>
       </c>
       <c r="R8" t="n">
-        <v>0.436</v>
+        <v>0.434</v>
       </c>
       <c r="S8" t="n">
-        <v>0.416</v>
+        <v>0.411</v>
       </c>
       <c r="T8" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="U8" t="n">
-        <v>0.016</v>
+        <v>0.018</v>
       </c>
       <c r="V8" t="n">
         <v>0.021</v>
       </c>
       <c r="W8" t="n">
+        <v>0.061</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>0.104</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>0.077</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>0.099</v>
+      </c>
+      <c r="AD8" t="n">
         <v>0.064</v>
       </c>
-      <c r="X8" t="n">
-        <v>0.048</v>
-      </c>
-      <c r="Y8" t="n">
-        <v>0.111</v>
-      </c>
-      <c r="Z8" t="n">
+      <c r="AE8" t="n">
         <v>0.079</v>
       </c>
-      <c r="AA8" t="n">
-        <v>0.117</v>
-      </c>
-      <c r="AB8" t="n">
-        <v>0.081</v>
-      </c>
-      <c r="AC8" t="n">
-        <v>0.103</v>
-      </c>
-      <c r="AD8" t="n">
-        <v>0.068</v>
-      </c>
-      <c r="AE8" t="n">
-        <v>0.08</v>
-      </c>
       <c r="AF8" t="n">
-        <v>0.042</v>
+        <v>0.045</v>
       </c>
       <c r="AG8" t="n">
-        <v>0.049</v>
+        <v>0.05</v>
       </c>
       <c r="AH8" t="n">
-        <v>0.025</v>
+        <v>0.031</v>
       </c>
       <c r="AI8" t="n">
-        <v>0.031</v>
+        <v>0.036</v>
       </c>
       <c r="AJ8" t="n">
-        <v>0.021</v>
+        <v>0.015</v>
       </c>
       <c r="AK8" t="n">
-        <v>0.014</v>
+        <v>0.013</v>
       </c>
       <c r="AL8" t="n">
         <v>0.008999999999999999</v>
       </c>
       <c r="AM8" t="n">
-        <v>0.007</v>
+        <v>0.011</v>
       </c>
       <c r="AN8" t="n">
-        <v>0.011</v>
+        <v>0.012</v>
       </c>
     </row>
     <row r="9">
@@ -1534,46 +1534,46 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>4.637</v>
+        <v>4.505</v>
       </c>
       <c r="F9" t="n">
-        <v>3.506</v>
+        <v>3.546</v>
       </c>
       <c r="G9" t="n">
-        <v>0.595</v>
+        <v>0.582</v>
       </c>
       <c r="H9" t="n">
-        <v>0.405</v>
+        <v>0.418</v>
       </c>
       <c r="I9" t="n">
-        <v>0.349</v>
+        <v>0.319</v>
       </c>
       <c r="J9" t="n">
-        <v>0.119</v>
+        <v>0.122</v>
       </c>
       <c r="K9" t="n">
-        <v>0.127</v>
+        <v>0.141</v>
       </c>
       <c r="L9" t="n">
-        <v>0.153</v>
+        <v>0.163</v>
       </c>
       <c r="M9" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.082</v>
       </c>
       <c r="N9" t="n">
-        <v>0.164</v>
+        <v>0.173</v>
       </c>
       <c r="O9" t="n">
-        <v>0.462</v>
+        <v>0.444</v>
       </c>
       <c r="P9" t="n">
-        <v>2.34</v>
+        <v>2.276</v>
       </c>
       <c r="Q9" t="n">
-        <v>1.782</v>
+        <v>1.761</v>
       </c>
       <c r="R9" t="n">
-        <v>0.484</v>
+        <v>0.486</v>
       </c>
       <c r="S9" t="n">
         <v>0.327</v>
@@ -1582,64 +1582,64 @@
         <v>0</v>
       </c>
       <c r="U9" t="n">
-        <v>0.023</v>
+        <v>0.024</v>
       </c>
       <c r="V9" t="n">
-        <v>0.027</v>
+        <v>0.025</v>
       </c>
       <c r="W9" t="n">
-        <v>0.078</v>
+        <v>0.067</v>
       </c>
       <c r="X9" t="n">
-        <v>0.062</v>
+        <v>0.068</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.104</v>
+        <v>0.12</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.082</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.11</v>
+        <v>0.114</v>
       </c>
       <c r="AB9" t="n">
-        <v>0.079</v>
+        <v>0.081</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.106</v>
+        <v>0.102</v>
       </c>
       <c r="AD9" t="n">
-        <v>0.068</v>
+        <v>0.058</v>
       </c>
       <c r="AE9" t="n">
-        <v>0.073</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="AF9" t="n">
-        <v>0.042</v>
+        <v>0.049</v>
       </c>
       <c r="AG9" t="n">
-        <v>0.047</v>
+        <v>0.04</v>
       </c>
       <c r="AH9" t="n">
-        <v>0.024</v>
+        <v>0.026</v>
       </c>
       <c r="AI9" t="n">
-        <v>0.026</v>
+        <v>0.022</v>
       </c>
       <c r="AJ9" t="n">
         <v>0.014</v>
       </c>
       <c r="AK9" t="n">
-        <v>0.013</v>
+        <v>0.012</v>
       </c>
       <c r="AL9" t="n">
-        <v>0.006</v>
+        <v>0.007</v>
       </c>
       <c r="AM9" t="n">
-        <v>0.006</v>
+        <v>0.004</v>
       </c>
       <c r="AN9" t="n">
-        <v>0.01</v>
+        <v>0.011</v>
       </c>
     </row>
     <row r="10">
@@ -1662,49 +1662,49 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>4.616</v>
+        <v>4.705</v>
       </c>
       <c r="F10" t="n">
-        <v>4.279</v>
+        <v>4.383</v>
       </c>
       <c r="G10" t="n">
-        <v>0.534</v>
+        <v>0.533</v>
       </c>
       <c r="H10" t="n">
-        <v>0.466</v>
+        <v>0.467</v>
       </c>
       <c r="I10" t="n">
-        <v>0.302</v>
+        <v>0.294</v>
       </c>
       <c r="J10" t="n">
-        <v>0.102</v>
+        <v>0.113</v>
       </c>
       <c r="K10" t="n">
-        <v>0.129</v>
+        <v>0.126</v>
       </c>
       <c r="L10" t="n">
-        <v>0.228</v>
+        <v>0.233</v>
       </c>
       <c r="M10" t="n">
-        <v>0.089</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="N10" t="n">
-        <v>0.15</v>
+        <v>0.148</v>
       </c>
       <c r="O10" t="n">
-        <v>0.52</v>
+        <v>0.507</v>
       </c>
       <c r="P10" t="n">
-        <v>2.623</v>
+        <v>2.665</v>
       </c>
       <c r="Q10" t="n">
-        <v>2.653</v>
+        <v>2.712</v>
       </c>
       <c r="R10" t="n">
-        <v>0.42</v>
+        <v>0.429</v>
       </c>
       <c r="S10" t="n">
-        <v>0.433</v>
+        <v>0.428</v>
       </c>
       <c r="T10" t="n">
         <v>0</v>
@@ -1713,61 +1713,61 @@
         <v>0.015</v>
       </c>
       <c r="V10" t="n">
-        <v>0.018</v>
+        <v>0.02</v>
       </c>
       <c r="W10" t="n">
-        <v>0.048</v>
+        <v>0.05</v>
       </c>
       <c r="X10" t="n">
         <v>0.043</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.105</v>
+        <v>0.097</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.081</v>
+        <v>0.073</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.118</v>
+        <v>0.096</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.082</v>
+        <v>0.078</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.105</v>
+        <v>0.109</v>
       </c>
       <c r="AD10" t="n">
         <v>0.065</v>
       </c>
       <c r="AE10" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.09</v>
       </c>
       <c r="AF10" t="n">
-        <v>0.051</v>
+        <v>0.057</v>
       </c>
       <c r="AG10" t="n">
-        <v>0.053</v>
+        <v>0.06</v>
       </c>
       <c r="AH10" t="n">
-        <v>0.039</v>
+        <v>0.033</v>
       </c>
       <c r="AI10" t="n">
-        <v>0.034</v>
+        <v>0.035</v>
       </c>
       <c r="AJ10" t="n">
         <v>0.023</v>
       </c>
       <c r="AK10" t="n">
-        <v>0.019</v>
+        <v>0.022</v>
       </c>
       <c r="AL10" t="n">
-        <v>0.012</v>
+        <v>0.01</v>
       </c>
       <c r="AM10" t="n">
         <v>0.007</v>
       </c>
       <c r="AN10" t="n">
-        <v>0.013</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="11">
@@ -1790,112 +1790,112 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>2.791</v>
+        <v>2.892</v>
       </c>
       <c r="F11" t="n">
-        <v>4.278</v>
+        <v>4.62</v>
       </c>
       <c r="G11" t="n">
-        <v>0.307</v>
+        <v>0.289</v>
       </c>
       <c r="H11" t="n">
-        <v>0.6929999999999999</v>
+        <v>0.711</v>
       </c>
       <c r="I11" t="n">
-        <v>0.118</v>
+        <v>0.113</v>
       </c>
       <c r="J11" t="n">
-        <v>0.077</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="K11" t="n">
-        <v>0.112</v>
+        <v>0.103</v>
       </c>
       <c r="L11" t="n">
-        <v>0.354</v>
+        <v>0.378</v>
       </c>
       <c r="M11" t="n">
-        <v>0.143</v>
+        <v>0.137</v>
       </c>
       <c r="N11" t="n">
         <v>0.196</v>
       </c>
       <c r="O11" t="n">
-        <v>0.412</v>
+        <v>0.447</v>
       </c>
       <c r="P11" t="n">
-        <v>1.408</v>
+        <v>1.447</v>
       </c>
       <c r="Q11" t="n">
-        <v>2.416</v>
+        <v>2.537</v>
       </c>
       <c r="R11" t="n">
-        <v>0.265</v>
+        <v>0.26</v>
       </c>
       <c r="S11" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="T11" t="n">
         <v>0</v>
       </c>
       <c r="U11" t="n">
-        <v>0.032</v>
+        <v>0.034</v>
       </c>
       <c r="V11" t="n">
-        <v>0.045</v>
+        <v>0.038</v>
       </c>
       <c r="W11" t="n">
-        <v>0.096</v>
+        <v>0.081</v>
       </c>
       <c r="X11" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.077</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.135</v>
+        <v>0.127</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.099</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.119</v>
+        <v>0.117</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.077</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.097</v>
       </c>
       <c r="AD11" t="n">
         <v>0.052</v>
       </c>
       <c r="AE11" t="n">
-        <v>0.053</v>
+        <v>0.057</v>
       </c>
       <c r="AF11" t="n">
         <v>0.035</v>
       </c>
       <c r="AG11" t="n">
-        <v>0.031</v>
+        <v>0.041</v>
       </c>
       <c r="AH11" t="n">
-        <v>0.017</v>
+        <v>0.026</v>
       </c>
       <c r="AI11" t="n">
-        <v>0.015</v>
+        <v>0.016</v>
       </c>
       <c r="AJ11" t="n">
-        <v>0.007</v>
+        <v>0.012</v>
       </c>
       <c r="AK11" t="n">
-        <v>0.01</v>
+        <v>0.011</v>
       </c>
       <c r="AL11" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="AM11" t="n">
         <v>0.003</v>
       </c>
       <c r="AN11" t="n">
-        <v>0.004</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="12">
@@ -1918,103 +1918,103 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>3.227</v>
+        <v>3.23</v>
       </c>
       <c r="F12" t="n">
-        <v>3.749</v>
+        <v>3.59</v>
       </c>
       <c r="G12" t="n">
-        <v>0.409</v>
+        <v>0.426</v>
       </c>
       <c r="H12" t="n">
-        <v>0.591</v>
+        <v>0.574</v>
       </c>
       <c r="I12" t="n">
-        <v>0.186</v>
+        <v>0.184</v>
       </c>
       <c r="J12" t="n">
-        <v>0.094</v>
+        <v>0.107</v>
       </c>
       <c r="K12" t="n">
-        <v>0.129</v>
+        <v>0.135</v>
       </c>
       <c r="L12" t="n">
-        <v>0.257</v>
+        <v>0.245</v>
       </c>
       <c r="M12" t="n">
-        <v>0.122</v>
+        <v>0.121</v>
       </c>
       <c r="N12" t="n">
-        <v>0.212</v>
+        <v>0.207</v>
       </c>
       <c r="O12" t="n">
-        <v>0.44</v>
+        <v>0.404</v>
       </c>
       <c r="P12" t="n">
-        <v>1.706</v>
+        <v>1.647</v>
       </c>
       <c r="Q12" t="n">
-        <v>2.108</v>
+        <v>1.977</v>
       </c>
       <c r="R12" t="n">
-        <v>0.35</v>
+        <v>0.354</v>
       </c>
       <c r="S12" t="n">
-        <v>0.465</v>
+        <v>0.451</v>
       </c>
       <c r="T12" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="U12" t="n">
-        <v>0.047</v>
+        <v>0.042</v>
       </c>
       <c r="V12" t="n">
-        <v>0.048</v>
+        <v>0.043</v>
       </c>
       <c r="W12" t="n">
-        <v>0.097</v>
+        <v>0.11</v>
       </c>
       <c r="X12" t="n">
-        <v>0.073</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.128</v>
+        <v>0.139</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.091</v>
+        <v>0.095</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.131</v>
+        <v>0.123</v>
       </c>
       <c r="AB12" t="n">
-        <v>0.077</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.082</v>
+        <v>0.081</v>
       </c>
       <c r="AD12" t="n">
-        <v>0.052</v>
+        <v>0.054</v>
       </c>
       <c r="AE12" t="n">
-        <v>0.056</v>
+        <v>0.055</v>
       </c>
       <c r="AF12" t="n">
-        <v>0.026</v>
+        <v>0.027</v>
       </c>
       <c r="AG12" t="n">
-        <v>0.036</v>
+        <v>0.027</v>
       </c>
       <c r="AH12" t="n">
-        <v>0.017</v>
+        <v>0.014</v>
       </c>
       <c r="AI12" t="n">
-        <v>0.016</v>
+        <v>0.014</v>
       </c>
       <c r="AJ12" t="n">
-        <v>0.007</v>
+        <v>0.006</v>
       </c>
       <c r="AK12" t="n">
-        <v>0.007</v>
+        <v>0.002</v>
       </c>
       <c r="AL12" t="n">
         <v>0.003</v>
@@ -2023,7 +2023,7 @@
         <v>0.002</v>
       </c>
       <c r="AN12" t="n">
-        <v>0.004</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="13">
@@ -2046,49 +2046,49 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>4.296</v>
+        <v>4.254</v>
       </c>
       <c r="F13" t="n">
-        <v>5.549</v>
+        <v>5.326</v>
       </c>
       <c r="G13" t="n">
-        <v>0.349</v>
+        <v>0.373</v>
       </c>
       <c r="H13" t="n">
-        <v>0.651</v>
+        <v>0.627</v>
       </c>
       <c r="I13" t="n">
-        <v>0.185</v>
+        <v>0.174</v>
       </c>
       <c r="J13" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>0.095</v>
+        <v>0.113</v>
       </c>
       <c r="L13" t="n">
-        <v>0.354</v>
+        <v>0.338</v>
       </c>
       <c r="M13" t="n">
-        <v>0.122</v>
+        <v>0.107</v>
       </c>
       <c r="N13" t="n">
-        <v>0.175</v>
+        <v>0.182</v>
       </c>
       <c r="O13" t="n">
-        <v>0.502</v>
+        <v>0.495</v>
       </c>
       <c r="P13" t="n">
-        <v>2.429</v>
+        <v>2.404</v>
       </c>
       <c r="Q13" t="n">
-        <v>3.152</v>
+        <v>3.025</v>
       </c>
       <c r="R13" t="n">
-        <v>0.339</v>
+        <v>0.366</v>
       </c>
       <c r="S13" t="n">
-        <v>0.523</v>
+        <v>0.491</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -2097,61 +2097,61 @@
         <v>0.011</v>
       </c>
       <c r="V13" t="n">
-        <v>0.012</v>
+        <v>0.01</v>
       </c>
       <c r="W13" t="n">
-        <v>0.037</v>
+        <v>0.044</v>
       </c>
       <c r="X13" t="n">
-        <v>0.043</v>
+        <v>0.036</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.074</v>
+        <v>0.077</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.066</v>
+        <v>0.062</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.097</v>
+        <v>0.116</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.074</v>
+        <v>0.078</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.099</v>
+        <v>0.114</v>
       </c>
       <c r="AD13" t="n">
-        <v>0.073</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="AE13" t="n">
-        <v>0.093</v>
+        <v>0.09</v>
       </c>
       <c r="AF13" t="n">
         <v>0.059</v>
       </c>
       <c r="AG13" t="n">
-        <v>0.066</v>
+        <v>0.063</v>
       </c>
       <c r="AH13" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="AI13" t="n">
         <v>0.041</v>
       </c>
-      <c r="AI13" t="n">
-        <v>0.042</v>
-      </c>
       <c r="AJ13" t="n">
-        <v>0.029</v>
+        <v>0.022</v>
       </c>
       <c r="AK13" t="n">
-        <v>0.027</v>
+        <v>0.024</v>
       </c>
       <c r="AL13" t="n">
-        <v>0.016</v>
+        <v>0.013</v>
       </c>
       <c r="AM13" t="n">
-        <v>0.012</v>
+        <v>0.013</v>
       </c>
       <c r="AN13" t="n">
-        <v>0.029</v>
+        <v>0.024</v>
       </c>
     </row>
     <row r="14">
@@ -2174,100 +2174,100 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>3.371</v>
+        <v>3.227</v>
       </c>
       <c r="F14" t="n">
-        <v>3.63</v>
+        <v>3.586</v>
       </c>
       <c r="G14" t="n">
-        <v>0.446</v>
+        <v>0.433</v>
       </c>
       <c r="H14" t="n">
-        <v>0.554</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="I14" t="n">
-        <v>0.215</v>
+        <v>0.194</v>
       </c>
       <c r="J14" t="n">
-        <v>0.095</v>
+        <v>0.1</v>
       </c>
       <c r="K14" t="n">
-        <v>0.136</v>
+        <v>0.14</v>
       </c>
       <c r="L14" t="n">
-        <v>0.238</v>
+        <v>0.239</v>
       </c>
       <c r="M14" t="n">
-        <v>0.123</v>
+        <v>0.125</v>
       </c>
       <c r="N14" t="n">
-        <v>0.194</v>
+        <v>0.203</v>
       </c>
       <c r="O14" t="n">
-        <v>0.382</v>
+        <v>0.388</v>
       </c>
       <c r="P14" t="n">
-        <v>1.62</v>
+        <v>1.524</v>
       </c>
       <c r="Q14" t="n">
-        <v>1.879</v>
+        <v>1.909</v>
       </c>
       <c r="R14" t="n">
-        <v>0.358</v>
+        <v>0.344</v>
       </c>
       <c r="S14" t="n">
-        <v>0.432</v>
+        <v>0.454</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
       </c>
       <c r="U14" t="n">
-        <v>0.039</v>
+        <v>0.049</v>
       </c>
       <c r="V14" t="n">
         <v>0.039</v>
       </c>
       <c r="W14" t="n">
-        <v>0.102</v>
+        <v>0.11</v>
       </c>
       <c r="X14" t="n">
-        <v>0.091</v>
+        <v>0.09</v>
       </c>
       <c r="Y14" t="n">
-        <v>0.128</v>
+        <v>0.126</v>
       </c>
       <c r="Z14" t="n">
-        <v>0.094</v>
+        <v>0.095</v>
       </c>
       <c r="AA14" t="n">
-        <v>0.118</v>
+        <v>0.124</v>
       </c>
       <c r="AB14" t="n">
-        <v>0.065</v>
+        <v>0.081</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.089</v>
+        <v>0.082</v>
       </c>
       <c r="AD14" t="n">
-        <v>0.054</v>
+        <v>0.05</v>
       </c>
       <c r="AE14" t="n">
-        <v>0.063</v>
+        <v>0.047</v>
       </c>
       <c r="AF14" t="n">
-        <v>0.034</v>
+        <v>0.025</v>
       </c>
       <c r="AG14" t="n">
-        <v>0.03</v>
+        <v>0.028</v>
       </c>
       <c r="AH14" t="n">
-        <v>0.019</v>
+        <v>0.016</v>
       </c>
       <c r="AI14" t="n">
-        <v>0.012</v>
+        <v>0.011</v>
       </c>
       <c r="AJ14" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.011</v>
       </c>
       <c r="AK14" t="n">
         <v>0.006</v>
@@ -2276,10 +2276,10 @@
         <v>0.003</v>
       </c>
       <c r="AM14" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="AN14" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="15">
@@ -2302,49 +2302,49 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>6.14</v>
+        <v>5.907</v>
       </c>
       <c r="F15" t="n">
-        <v>6.566</v>
+        <v>6.238</v>
       </c>
       <c r="G15" t="n">
-        <v>0.441</v>
+        <v>0.456</v>
       </c>
       <c r="H15" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.544</v>
       </c>
       <c r="I15" t="n">
-        <v>0.281</v>
+        <v>0.282</v>
       </c>
       <c r="J15" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.078</v>
       </c>
       <c r="K15" t="n">
-        <v>0.089</v>
+        <v>0.096</v>
       </c>
       <c r="L15" t="n">
-        <v>0.315</v>
+        <v>0.304</v>
       </c>
       <c r="M15" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.091</v>
       </c>
       <c r="N15" t="n">
-        <v>0.156</v>
+        <v>0.149</v>
       </c>
       <c r="O15" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.5629999999999999</v>
       </c>
       <c r="P15" t="n">
-        <v>3.161</v>
+        <v>3.106</v>
       </c>
       <c r="Q15" t="n">
-        <v>3.614</v>
+        <v>3.418</v>
       </c>
       <c r="R15" t="n">
-        <v>0.402</v>
+        <v>0.403</v>
       </c>
       <c r="S15" t="n">
-        <v>0.482</v>
+        <v>0.473</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -2353,61 +2353,61 @@
         <v>0.003</v>
       </c>
       <c r="V15" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="W15" t="n">
-        <v>0.017</v>
+        <v>0.016</v>
       </c>
       <c r="X15" t="n">
-        <v>0.015</v>
+        <v>0.023</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.035</v>
+        <v>0.041</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.06</v>
+        <v>0.075</v>
       </c>
       <c r="AB15" t="n">
-        <v>0.052</v>
+        <v>0.061</v>
       </c>
       <c r="AC15" t="n">
         <v>0.08599999999999999</v>
       </c>
       <c r="AD15" t="n">
-        <v>0.067</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="AE15" t="n">
-        <v>0.089</v>
+        <v>0.09</v>
       </c>
       <c r="AF15" t="n">
-        <v>0.062</v>
+        <v>0.06</v>
       </c>
       <c r="AG15" t="n">
-        <v>0.082</v>
+        <v>0.077</v>
       </c>
       <c r="AH15" t="n">
         <v>0.052</v>
       </c>
       <c r="AI15" t="n">
-        <v>0.073</v>
+        <v>0.067</v>
       </c>
       <c r="AJ15" t="n">
-        <v>0.049</v>
+        <v>0.041</v>
       </c>
       <c r="AK15" t="n">
-        <v>0.052</v>
+        <v>0.044</v>
       </c>
       <c r="AL15" t="n">
-        <v>0.03</v>
+        <v>0.031</v>
       </c>
       <c r="AM15" t="n">
-        <v>0.033</v>
+        <v>0.031</v>
       </c>
       <c r="AN15" t="n">
-        <v>0.109</v>
+        <v>0.091</v>
       </c>
     </row>
     <row r="16">
@@ -2430,112 +2430,112 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>3.702</v>
+        <v>3.666</v>
       </c>
       <c r="F16" t="n">
-        <v>4.074</v>
+        <v>4.101</v>
       </c>
       <c r="G16" t="n">
-        <v>0.427</v>
+        <v>0.43</v>
       </c>
       <c r="H16" t="n">
-        <v>0.573</v>
+        <v>0.57</v>
       </c>
       <c r="I16" t="n">
-        <v>0.212</v>
+        <v>0.21</v>
       </c>
       <c r="J16" t="n">
-        <v>0.094</v>
+        <v>0.095</v>
       </c>
       <c r="K16" t="n">
-        <v>0.121</v>
+        <v>0.125</v>
       </c>
       <c r="L16" t="n">
-        <v>0.268</v>
+        <v>0.273</v>
       </c>
       <c r="M16" t="n">
-        <v>0.11</v>
+        <v>0.113</v>
       </c>
       <c r="N16" t="n">
-        <v>0.195</v>
+        <v>0.184</v>
       </c>
       <c r="O16" t="n">
-        <v>0.451</v>
+        <v>0.461</v>
       </c>
       <c r="P16" t="n">
-        <v>1.987</v>
+        <v>1.968</v>
       </c>
       <c r="Q16" t="n">
-        <v>2.314</v>
+        <v>2.361</v>
       </c>
       <c r="R16" t="n">
-        <v>0.379</v>
+        <v>0.363</v>
       </c>
       <c r="S16" t="n">
-        <v>0.46</v>
+        <v>0.475</v>
       </c>
       <c r="T16" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="U16" t="n">
         <v>0.029</v>
       </c>
       <c r="V16" t="n">
-        <v>0.02</v>
+        <v>0.028</v>
       </c>
       <c r="W16" t="n">
-        <v>0.075</v>
+        <v>0.076</v>
       </c>
       <c r="X16" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.066</v>
       </c>
       <c r="Y16" t="n">
-        <v>0.126</v>
+        <v>0.108</v>
       </c>
       <c r="Z16" t="n">
-        <v>0.083</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="AA16" t="n">
-        <v>0.127</v>
+        <v>0.137</v>
       </c>
       <c r="AB16" t="n">
-        <v>0.078</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="AC16" t="n">
-        <v>0.103</v>
+        <v>0.095</v>
       </c>
       <c r="AD16" t="n">
-        <v>0.066</v>
+        <v>0.068</v>
       </c>
       <c r="AE16" t="n">
-        <v>0.064</v>
+        <v>0.067</v>
       </c>
       <c r="AF16" t="n">
-        <v>0.034</v>
+        <v>0.038</v>
       </c>
       <c r="AG16" t="n">
-        <v>0.039</v>
+        <v>0.036</v>
       </c>
       <c r="AH16" t="n">
-        <v>0.025</v>
+        <v>0.018</v>
       </c>
       <c r="AI16" t="n">
         <v>0.019</v>
       </c>
       <c r="AJ16" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="AK16" t="n">
         <v>0.011</v>
-      </c>
-      <c r="AK16" t="n">
-        <v>0.014</v>
       </c>
       <c r="AL16" t="n">
         <v>0.006</v>
       </c>
       <c r="AM16" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
       <c r="AN16" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: portfolio selection fallback — supplement shortfall with top-ranked candidates, dashboard picks upload file with most lineups
</commit_message>
<xml_diff>
--- a/data/live/BallparkPal_Games_2026-04-12.xlsx
+++ b/data/live/BallparkPal_Games_2026-04-12.xlsx
@@ -620,7 +620,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>822998</v>
+        <v>822828</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -629,118 +629,118 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TB </t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>4.505</v>
+        <v>4.593</v>
       </c>
       <c r="F2" t="n">
-        <v>3.546</v>
+        <v>3.94</v>
       </c>
       <c r="G2" t="n">
-        <v>0.582</v>
+        <v>0.54</v>
       </c>
       <c r="H2" t="n">
-        <v>0.418</v>
+        <v>0.46</v>
       </c>
       <c r="I2" t="n">
-        <v>0.319</v>
+        <v>0.302</v>
       </c>
       <c r="J2" t="n">
-        <v>0.122</v>
+        <v>0.096</v>
       </c>
       <c r="K2" t="n">
-        <v>0.141</v>
+        <v>0.142</v>
       </c>
       <c r="L2" t="n">
-        <v>0.163</v>
+        <v>0.175</v>
       </c>
       <c r="M2" t="n">
-        <v>0.082</v>
+        <v>0.097</v>
       </c>
       <c r="N2" t="n">
-        <v>0.173</v>
+        <v>0.188</v>
       </c>
       <c r="O2" t="n">
-        <v>0.444</v>
+        <v>0.489</v>
       </c>
       <c r="P2" t="n">
-        <v>2.276</v>
+        <v>2.835</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.761</v>
+        <v>2.115</v>
       </c>
       <c r="R2" t="n">
-        <v>0.486</v>
+        <v>0.521</v>
       </c>
       <c r="S2" t="n">
-        <v>0.327</v>
+        <v>0.331</v>
       </c>
       <c r="T2" t="n">
         <v>0</v>
       </c>
       <c r="U2" t="n">
-        <v>0.024</v>
+        <v>0.021</v>
       </c>
       <c r="V2" t="n">
-        <v>0.025</v>
+        <v>0.016</v>
       </c>
       <c r="W2" t="n">
-        <v>0.067</v>
+        <v>0.064</v>
       </c>
       <c r="X2" t="n">
-        <v>0.068</v>
+        <v>0.048</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.12</v>
+        <v>0.105</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.081</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.114</v>
+        <v>0.115</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.081</v>
+        <v>0.077</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.102</v>
+        <v>0.104</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.058</v>
+        <v>0.074</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.049</v>
+        <v>0.046</v>
       </c>
       <c r="AG2" t="n">
-        <v>0.04</v>
+        <v>0.051</v>
       </c>
       <c r="AH2" t="n">
-        <v>0.026</v>
+        <v>0.027</v>
       </c>
       <c r="AI2" t="n">
-        <v>0.022</v>
+        <v>0.03</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0.014</v>
+        <v>0.015</v>
       </c>
       <c r="AK2" t="n">
-        <v>0.012</v>
+        <v>0.015</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.007</v>
+        <v>0.005</v>
       </c>
       <c r="AM2" t="n">
-        <v>0.004</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="AN2" t="n">
         <v>0.011</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>823075</v>
+        <v>823154</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -757,126 +757,126 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>HOU</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>4.705</v>
+        <v>3.941</v>
       </c>
       <c r="F3" t="n">
-        <v>4.383</v>
+        <v>4.426</v>
       </c>
       <c r="G3" t="n">
-        <v>0.533</v>
+        <v>0.426</v>
       </c>
       <c r="H3" t="n">
-        <v>0.467</v>
+        <v>0.574</v>
       </c>
       <c r="I3" t="n">
-        <v>0.294</v>
+        <v>0.21</v>
       </c>
       <c r="J3" t="n">
-        <v>0.113</v>
+        <v>0.089</v>
       </c>
       <c r="K3" t="n">
-        <v>0.126</v>
+        <v>0.127</v>
       </c>
       <c r="L3" t="n">
-        <v>0.233</v>
+        <v>0.279</v>
       </c>
       <c r="M3" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.11</v>
       </c>
       <c r="N3" t="n">
-        <v>0.148</v>
+        <v>0.186</v>
       </c>
       <c r="O3" t="n">
-        <v>0.507</v>
+        <v>0.471</v>
       </c>
       <c r="P3" t="n">
-        <v>2.665</v>
+        <v>2.023</v>
       </c>
       <c r="Q3" t="n">
-        <v>2.712</v>
+        <v>2.513</v>
       </c>
       <c r="R3" t="n">
-        <v>0.429</v>
+        <v>0.353</v>
       </c>
       <c r="S3" t="n">
-        <v>0.428</v>
+        <v>0.482</v>
       </c>
       <c r="T3" t="n">
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>0.015</v>
+        <v>0.023</v>
       </c>
       <c r="V3" t="n">
-        <v>0.02</v>
+        <v>0.017</v>
       </c>
       <c r="W3" t="n">
-        <v>0.05</v>
+        <v>0.065</v>
       </c>
       <c r="X3" t="n">
-        <v>0.043</v>
+        <v>0.056</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.097</v>
+        <v>0.107</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.073</v>
+        <v>0.079</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.096</v>
+        <v>0.117</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.078</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="AC3" t="n">
         <v>0.109</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.065</v>
+        <v>0.062</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.09</v>
+        <v>0.079</v>
       </c>
       <c r="AF3" t="n">
-        <v>0.057</v>
+        <v>0.042</v>
       </c>
       <c r="AG3" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="AH3" t="n">
-        <v>0.033</v>
+        <v>0.027</v>
       </c>
       <c r="AI3" t="n">
-        <v>0.035</v>
+        <v>0.024</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0.023</v>
+        <v>0.017</v>
       </c>
       <c r="AK3" t="n">
-        <v>0.022</v>
+        <v>0.014</v>
       </c>
       <c r="AL3" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="AN3" t="n">
         <v>0.01</v>
-      </c>
-      <c r="AM3" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="AN3" t="n">
-        <v>0.017</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>823317</v>
+        <v>823479</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -885,126 +885,126 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>ARI</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">SD </t>
+          <t>PHI</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>2.892</v>
+        <v>4.257</v>
       </c>
       <c r="F4" t="n">
-        <v>4.62</v>
+        <v>4.543</v>
       </c>
       <c r="G4" t="n">
-        <v>0.289</v>
+        <v>0.436</v>
       </c>
       <c r="H4" t="n">
-        <v>0.711</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="I4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.079</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.106</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="M4" t="n">
         <v>0.113</v>
       </c>
-      <c r="J4" t="n">
-        <v>0.07199999999999999</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.103</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.378</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.137</v>
-      </c>
       <c r="N4" t="n">
-        <v>0.196</v>
+        <v>0.184</v>
       </c>
       <c r="O4" t="n">
-        <v>0.447</v>
+        <v>0.481</v>
       </c>
       <c r="P4" t="n">
-        <v>1.447</v>
+        <v>2.339</v>
       </c>
       <c r="Q4" t="n">
-        <v>2.537</v>
+        <v>2.536</v>
       </c>
       <c r="R4" t="n">
-        <v>0.26</v>
+        <v>0.401</v>
       </c>
       <c r="S4" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.452</v>
       </c>
       <c r="T4" t="n">
         <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>0.034</v>
+        <v>0.015</v>
       </c>
       <c r="V4" t="n">
-        <v>0.038</v>
+        <v>0.019</v>
       </c>
       <c r="W4" t="n">
-        <v>0.081</v>
+        <v>0.064</v>
       </c>
       <c r="X4" t="n">
-        <v>0.077</v>
+        <v>0.053</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.127</v>
+        <v>0.1</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.117</v>
+        <v>0.109</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.077</v>
+        <v>0.08</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.097</v>
+        <v>0.105</v>
       </c>
       <c r="AD4" t="n">
-        <v>0.052</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="AE4" t="n">
-        <v>0.057</v>
+        <v>0.075</v>
       </c>
       <c r="AF4" t="n">
-        <v>0.035</v>
+        <v>0.053</v>
       </c>
       <c r="AG4" t="n">
-        <v>0.041</v>
+        <v>0.049</v>
       </c>
       <c r="AH4" t="n">
-        <v>0.026</v>
+        <v>0.031</v>
       </c>
       <c r="AI4" t="n">
-        <v>0.016</v>
+        <v>0.031</v>
       </c>
       <c r="AJ4" t="n">
-        <v>0.012</v>
+        <v>0.021</v>
       </c>
       <c r="AK4" t="n">
-        <v>0.011</v>
+        <v>0.018</v>
       </c>
       <c r="AL4" t="n">
-        <v>0.004</v>
+        <v>0.01</v>
       </c>
       <c r="AM4" t="n">
-        <v>0.003</v>
+        <v>0.006</v>
       </c>
       <c r="AN4" t="n">
-        <v>0.008</v>
+        <v>0.019</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>823642</v>
+        <v>823804</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1013,126 +1013,126 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ATH</t>
+          <t>WAS</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>NYM</t>
+          <t>MIL</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>3.23</v>
+        <v>3.667</v>
       </c>
       <c r="F5" t="n">
-        <v>3.59</v>
+        <v>4.673</v>
       </c>
       <c r="G5" t="n">
-        <v>0.426</v>
+        <v>0.372</v>
       </c>
       <c r="H5" t="n">
-        <v>0.574</v>
+        <v>0.628</v>
       </c>
       <c r="I5" t="n">
-        <v>0.184</v>
+        <v>0.179</v>
       </c>
       <c r="J5" t="n">
-        <v>0.107</v>
+        <v>0.076</v>
       </c>
       <c r="K5" t="n">
-        <v>0.135</v>
+        <v>0.117</v>
       </c>
       <c r="L5" t="n">
-        <v>0.245</v>
+        <v>0.326</v>
       </c>
       <c r="M5" t="n">
-        <v>0.121</v>
+        <v>0.129</v>
       </c>
       <c r="N5" t="n">
-        <v>0.207</v>
+        <v>0.173</v>
       </c>
       <c r="O5" t="n">
-        <v>0.404</v>
+        <v>0.477</v>
       </c>
       <c r="P5" t="n">
-        <v>1.647</v>
+        <v>1.899</v>
       </c>
       <c r="Q5" t="n">
-        <v>1.977</v>
+        <v>2.565</v>
       </c>
       <c r="R5" t="n">
-        <v>0.354</v>
+        <v>0.332</v>
       </c>
       <c r="S5" t="n">
-        <v>0.451</v>
+        <v>0.501</v>
       </c>
       <c r="T5" t="n">
         <v>0</v>
       </c>
       <c r="U5" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0.057</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0.106</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0.081</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>0.111</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>0.083</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>0.106</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>0.077</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="AG5" t="n">
         <v>0.042</v>
       </c>
-      <c r="V5" t="n">
-        <v>0.043</v>
-      </c>
-      <c r="W5" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="X5" t="n">
-        <v>0.08500000000000001</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>0.139</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>0.095</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>0.123</v>
-      </c>
-      <c r="AB5" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="AC5" t="n">
-        <v>0.081</v>
-      </c>
-      <c r="AD5" t="n">
-        <v>0.054</v>
-      </c>
-      <c r="AE5" t="n">
-        <v>0.055</v>
-      </c>
-      <c r="AF5" t="n">
-        <v>0.027</v>
-      </c>
-      <c r="AG5" t="n">
-        <v>0.027</v>
-      </c>
       <c r="AH5" t="n">
-        <v>0.014</v>
+        <v>0.029</v>
       </c>
       <c r="AI5" t="n">
-        <v>0.014</v>
+        <v>0.025</v>
       </c>
       <c r="AJ5" t="n">
-        <v>0.006</v>
+        <v>0.015</v>
       </c>
       <c r="AK5" t="n">
-        <v>0.002</v>
+        <v>0.012</v>
       </c>
       <c r="AL5" t="n">
-        <v>0.003</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="AM5" t="n">
-        <v>0.002</v>
+        <v>0.007</v>
       </c>
       <c r="AN5" t="n">
-        <v>0.006</v>
+        <v>0.012</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>824126</v>
+        <v>823966</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1141,126 +1141,126 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CHW</t>
+          <t>TEX</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">KC </t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>4.254</v>
+        <v>4.783</v>
       </c>
       <c r="F6" t="n">
-        <v>5.326</v>
+        <v>3.687</v>
       </c>
       <c r="G6" t="n">
-        <v>0.373</v>
+        <v>0.579</v>
       </c>
       <c r="H6" t="n">
-        <v>0.627</v>
+        <v>0.421</v>
       </c>
       <c r="I6" t="n">
-        <v>0.174</v>
+        <v>0.33</v>
       </c>
       <c r="J6" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.118</v>
       </c>
       <c r="K6" t="n">
-        <v>0.113</v>
+        <v>0.131</v>
       </c>
       <c r="L6" t="n">
-        <v>0.338</v>
+        <v>0.158</v>
       </c>
       <c r="M6" t="n">
-        <v>0.107</v>
+        <v>0.081</v>
       </c>
       <c r="N6" t="n">
         <v>0.182</v>
       </c>
       <c r="O6" t="n">
-        <v>0.495</v>
+        <v>0.498</v>
       </c>
       <c r="P6" t="n">
-        <v>2.404</v>
+        <v>2.799</v>
       </c>
       <c r="Q6" t="n">
-        <v>3.025</v>
+        <v>1.852</v>
       </c>
       <c r="R6" t="n">
-        <v>0.366</v>
+        <v>0.541</v>
       </c>
       <c r="S6" t="n">
-        <v>0.491</v>
+        <v>0.293</v>
       </c>
       <c r="T6" t="n">
         <v>0</v>
       </c>
       <c r="U6" t="n">
-        <v>0.011</v>
+        <v>0.016</v>
       </c>
       <c r="V6" t="n">
-        <v>0.01</v>
+        <v>0.019</v>
       </c>
       <c r="W6" t="n">
-        <v>0.044</v>
+        <v>0.067</v>
       </c>
       <c r="X6" t="n">
-        <v>0.036</v>
+        <v>0.055</v>
       </c>
       <c r="Y6" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0.127</v>
+      </c>
+      <c r="AB6" t="n">
         <v>0.077</v>
       </c>
-      <c r="Z6" t="n">
-        <v>0.062</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="AB6" t="n">
-        <v>0.078</v>
-      </c>
       <c r="AC6" t="n">
-        <v>0.114</v>
+        <v>0.109</v>
       </c>
       <c r="AD6" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.061</v>
       </c>
       <c r="AE6" t="n">
-        <v>0.09</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="AF6" t="n">
-        <v>0.059</v>
+        <v>0.048</v>
       </c>
       <c r="AG6" t="n">
-        <v>0.063</v>
+        <v>0.053</v>
       </c>
       <c r="AH6" t="n">
-        <v>0.034</v>
+        <v>0.03</v>
       </c>
       <c r="AI6" t="n">
-        <v>0.041</v>
+        <v>0.03</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0.022</v>
+        <v>0.015</v>
       </c>
       <c r="AK6" t="n">
-        <v>0.024</v>
+        <v>0.013</v>
       </c>
       <c r="AL6" t="n">
-        <v>0.013</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="AM6" t="n">
-        <v>0.013</v>
+        <v>0.005</v>
       </c>
       <c r="AN6" t="n">
-        <v>0.024</v>
+        <v>0.012</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>824293</v>
+        <v>824533</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1269,126 +1269,126 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>LAA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>CIN</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>3.227</v>
+        <v>3.95</v>
       </c>
       <c r="F7" t="n">
-        <v>3.586</v>
+        <v>4.212</v>
       </c>
       <c r="G7" t="n">
-        <v>0.433</v>
+        <v>0.456</v>
       </c>
       <c r="H7" t="n">
-        <v>0.5669999999999999</v>
+        <v>0.544</v>
       </c>
       <c r="I7" t="n">
-        <v>0.194</v>
+        <v>0.22</v>
       </c>
       <c r="J7" t="n">
-        <v>0.1</v>
+        <v>0.098</v>
       </c>
       <c r="K7" t="n">
-        <v>0.14</v>
+        <v>0.138</v>
       </c>
       <c r="L7" t="n">
-        <v>0.239</v>
+        <v>0.242</v>
       </c>
       <c r="M7" t="n">
-        <v>0.125</v>
+        <v>0.099</v>
       </c>
       <c r="N7" t="n">
         <v>0.203</v>
       </c>
       <c r="O7" t="n">
-        <v>0.388</v>
+        <v>0.447</v>
       </c>
       <c r="P7" t="n">
-        <v>1.524</v>
+        <v>2.002</v>
       </c>
       <c r="Q7" t="n">
-        <v>1.909</v>
+        <v>2.257</v>
       </c>
       <c r="R7" t="n">
-        <v>0.344</v>
+        <v>0.385</v>
       </c>
       <c r="S7" t="n">
-        <v>0.454</v>
+        <v>0.445</v>
       </c>
       <c r="T7" t="n">
         <v>0</v>
       </c>
       <c r="U7" t="n">
-        <v>0.049</v>
+        <v>0.019</v>
       </c>
       <c r="V7" t="n">
-        <v>0.039</v>
+        <v>0.028</v>
       </c>
       <c r="W7" t="n">
-        <v>0.11</v>
+        <v>0.078</v>
       </c>
       <c r="X7" t="n">
-        <v>0.09</v>
+        <v>0.062</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.126</v>
+        <v>0.119</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.095</v>
+        <v>0.075</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.124</v>
+        <v>0.127</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.081</v>
+        <v>0.064</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.082</v>
+        <v>0.105</v>
       </c>
       <c r="AD7" t="n">
-        <v>0.05</v>
+        <v>0.063</v>
       </c>
       <c r="AE7" t="n">
-        <v>0.047</v>
+        <v>0.067</v>
       </c>
       <c r="AF7" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="AH7" t="n">
         <v>0.025</v>
       </c>
-      <c r="AG7" t="n">
+      <c r="AI7" t="n">
         <v>0.028</v>
       </c>
-      <c r="AH7" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="AI7" t="n">
-        <v>0.011</v>
-      </c>
       <c r="AJ7" t="n">
-        <v>0.011</v>
+        <v>0.018</v>
       </c>
       <c r="AK7" t="n">
-        <v>0.006</v>
+        <v>0.02</v>
       </c>
       <c r="AL7" t="n">
-        <v>0.003</v>
+        <v>0.008</v>
       </c>
       <c r="AM7" t="n">
-        <v>0.003</v>
+        <v>0.005</v>
       </c>
       <c r="AN7" t="n">
-        <v>0.004</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>824696</v>
+        <v>824859</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1397,126 +1397,126 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t xml:space="preserve">SF </t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>BAL</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>5.675</v>
+        <v>4.255</v>
       </c>
       <c r="F8" t="n">
-        <v>5.776</v>
+        <v>4.267</v>
       </c>
       <c r="G8" t="n">
-        <v>0.484</v>
+        <v>0.483</v>
       </c>
       <c r="H8" t="n">
-        <v>0.516</v>
+        <v>0.517</v>
       </c>
       <c r="I8" t="n">
-        <v>0.277</v>
+        <v>0.261</v>
       </c>
       <c r="J8" t="n">
-        <v>0.095</v>
+        <v>0.102</v>
       </c>
       <c r="K8" t="n">
-        <v>0.112</v>
+        <v>0.12</v>
       </c>
       <c r="L8" t="n">
-        <v>0.277</v>
+        <v>0.249</v>
       </c>
       <c r="M8" t="n">
-        <v>0.093</v>
+        <v>0.1</v>
       </c>
       <c r="N8" t="n">
-        <v>0.147</v>
+        <v>0.169</v>
       </c>
       <c r="O8" t="n">
-        <v>0.541</v>
+        <v>0.49</v>
       </c>
       <c r="P8" t="n">
-        <v>2.948</v>
+        <v>2.478</v>
       </c>
       <c r="Q8" t="n">
-        <v>3.095</v>
+        <v>2.378</v>
       </c>
       <c r="R8" t="n">
-        <v>0.439</v>
+        <v>0.442</v>
       </c>
       <c r="S8" t="n">
-        <v>0.433</v>
+        <v>0.411</v>
       </c>
       <c r="T8" t="n">
         <v>0</v>
       </c>
       <c r="U8" t="n">
-        <v>0.005</v>
+        <v>0.016</v>
       </c>
       <c r="V8" t="n">
-        <v>0.005</v>
+        <v>0.018</v>
       </c>
       <c r="W8" t="n">
-        <v>0.016</v>
+        <v>0.053</v>
       </c>
       <c r="X8" t="n">
-        <v>0.023</v>
+        <v>0.061</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.053</v>
+        <v>0.098</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.055</v>
+        <v>0.09</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.082</v>
+        <v>0.121</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.062</v>
+        <v>0.089</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.104</v>
       </c>
       <c r="AD8" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.066</v>
       </c>
       <c r="AE8" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.074</v>
       </c>
       <c r="AF8" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.046</v>
       </c>
       <c r="AG8" t="n">
-        <v>0.073</v>
+        <v>0.048</v>
       </c>
       <c r="AH8" t="n">
-        <v>0.051</v>
+        <v>0.03</v>
       </c>
       <c r="AI8" t="n">
-        <v>0.063</v>
+        <v>0.027</v>
       </c>
       <c r="AJ8" t="n">
-        <v>0.041</v>
+        <v>0.014</v>
       </c>
       <c r="AK8" t="n">
-        <v>0.042</v>
+        <v>0.017</v>
       </c>
       <c r="AL8" t="n">
-        <v>0.024</v>
+        <v>0.01</v>
       </c>
       <c r="AM8" t="n">
-        <v>0.026</v>
+        <v>0.007</v>
       </c>
       <c r="AN8" t="n">
-        <v>0.065</v>
+        <v>0.012</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>824938</v>
+        <v>822998</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1525,126 +1525,126 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>NYY</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t xml:space="preserve">TB </t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>3.666</v>
+        <v>4.505</v>
       </c>
       <c r="F9" t="n">
-        <v>4.101</v>
+        <v>3.546</v>
       </c>
       <c r="G9" t="n">
-        <v>0.43</v>
+        <v>0.582</v>
       </c>
       <c r="H9" t="n">
-        <v>0.57</v>
+        <v>0.418</v>
       </c>
       <c r="I9" t="n">
-        <v>0.21</v>
+        <v>0.319</v>
       </c>
       <c r="J9" t="n">
-        <v>0.095</v>
+        <v>0.122</v>
       </c>
       <c r="K9" t="n">
-        <v>0.125</v>
+        <v>0.141</v>
       </c>
       <c r="L9" t="n">
-        <v>0.273</v>
+        <v>0.163</v>
       </c>
       <c r="M9" t="n">
-        <v>0.113</v>
+        <v>0.082</v>
       </c>
       <c r="N9" t="n">
-        <v>0.184</v>
+        <v>0.173</v>
       </c>
       <c r="O9" t="n">
-        <v>0.461</v>
+        <v>0.444</v>
       </c>
       <c r="P9" t="n">
-        <v>1.968</v>
+        <v>2.276</v>
       </c>
       <c r="Q9" t="n">
-        <v>2.361</v>
+        <v>1.761</v>
       </c>
       <c r="R9" t="n">
-        <v>0.363</v>
+        <v>0.486</v>
       </c>
       <c r="S9" t="n">
-        <v>0.475</v>
+        <v>0.327</v>
       </c>
       <c r="T9" t="n">
         <v>0</v>
       </c>
       <c r="U9" t="n">
-        <v>0.029</v>
+        <v>0.024</v>
       </c>
       <c r="V9" t="n">
-        <v>0.028</v>
+        <v>0.025</v>
       </c>
       <c r="W9" t="n">
-        <v>0.076</v>
+        <v>0.067</v>
       </c>
       <c r="X9" t="n">
-        <v>0.066</v>
+        <v>0.068</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.108</v>
+        <v>0.12</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.137</v>
+        <v>0.114</v>
       </c>
       <c r="AB9" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.081</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.095</v>
+        <v>0.102</v>
       </c>
       <c r="AD9" t="n">
-        <v>0.068</v>
+        <v>0.058</v>
       </c>
       <c r="AE9" t="n">
-        <v>0.067</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="AF9" t="n">
-        <v>0.038</v>
+        <v>0.049</v>
       </c>
       <c r="AG9" t="n">
-        <v>0.036</v>
+        <v>0.04</v>
       </c>
       <c r="AH9" t="n">
-        <v>0.018</v>
+        <v>0.026</v>
       </c>
       <c r="AI9" t="n">
-        <v>0.019</v>
+        <v>0.022</v>
       </c>
       <c r="AJ9" t="n">
-        <v>0.015</v>
+        <v>0.014</v>
       </c>
       <c r="AK9" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="AN9" t="n">
         <v>0.011</v>
-      </c>
-      <c r="AL9" t="n">
-        <v>0.006</v>
-      </c>
-      <c r="AM9" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="AN9" t="n">
-        <v>0.005</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>822828</v>
+        <v>823075</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1653,126 +1653,126 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>4.793</v>
+        <v>4.705</v>
       </c>
       <c r="F10" t="n">
-        <v>4.147</v>
+        <v>4.383</v>
       </c>
       <c r="G10" t="n">
-        <v>0.541</v>
+        <v>0.533</v>
       </c>
       <c r="H10" t="n">
-        <v>0.459</v>
+        <v>0.467</v>
       </c>
       <c r="I10" t="n">
-        <v>0.303</v>
+        <v>0.294</v>
       </c>
       <c r="J10" t="n">
-        <v>0.104</v>
+        <v>0.113</v>
       </c>
       <c r="K10" t="n">
-        <v>0.135</v>
+        <v>0.126</v>
       </c>
       <c r="L10" t="n">
-        <v>0.188</v>
+        <v>0.233</v>
       </c>
       <c r="M10" t="n">
-        <v>0.096</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="N10" t="n">
-        <v>0.175</v>
+        <v>0.148</v>
       </c>
       <c r="O10" t="n">
-        <v>0.502</v>
+        <v>0.507</v>
       </c>
       <c r="P10" t="n">
-        <v>2.884</v>
+        <v>2.665</v>
       </c>
       <c r="Q10" t="n">
-        <v>2.277</v>
+        <v>2.712</v>
       </c>
       <c r="R10" t="n">
-        <v>0.507</v>
+        <v>0.429</v>
       </c>
       <c r="S10" t="n">
-        <v>0.344</v>
+        <v>0.428</v>
       </c>
       <c r="T10" t="n">
         <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>0.013</v>
+        <v>0.015</v>
       </c>
       <c r="V10" t="n">
-        <v>0.017</v>
+        <v>0.02</v>
       </c>
       <c r="W10" t="n">
         <v>0.05</v>
       </c>
       <c r="X10" t="n">
-        <v>0.039</v>
+        <v>0.043</v>
       </c>
       <c r="Y10" t="n">
+        <v>0.097</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="AA10" t="n">
         <v>0.096</v>
       </c>
-      <c r="Z10" t="n">
-        <v>0.075</v>
-      </c>
-      <c r="AA10" t="n">
-        <v>0.124</v>
-      </c>
       <c r="AB10" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.078</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.108</v>
+        <v>0.109</v>
       </c>
       <c r="AD10" t="n">
         <v>0.065</v>
       </c>
       <c r="AE10" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.09</v>
       </c>
       <c r="AF10" t="n">
-        <v>0.055</v>
+        <v>0.057</v>
       </c>
       <c r="AG10" t="n">
-        <v>0.052</v>
+        <v>0.06</v>
       </c>
       <c r="AH10" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="AI10" t="n">
         <v>0.035</v>
       </c>
-      <c r="AI10" t="n">
-        <v>0.031</v>
-      </c>
       <c r="AJ10" t="n">
-        <v>0.021</v>
+        <v>0.023</v>
       </c>
       <c r="AK10" t="n">
-        <v>0.014</v>
+        <v>0.022</v>
       </c>
       <c r="AL10" t="n">
         <v>0.01</v>
       </c>
       <c r="AM10" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.007</v>
       </c>
       <c r="AN10" t="n">
-        <v>0.014</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>823154</v>
+        <v>823317</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1781,126 +1781,126 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>HOU</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t xml:space="preserve">SD </t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>3.941</v>
+        <v>2.892</v>
       </c>
       <c r="F11" t="n">
-        <v>4.426</v>
+        <v>4.62</v>
       </c>
       <c r="G11" t="n">
-        <v>0.426</v>
+        <v>0.289</v>
       </c>
       <c r="H11" t="n">
-        <v>0.574</v>
+        <v>0.711</v>
       </c>
       <c r="I11" t="n">
-        <v>0.21</v>
+        <v>0.113</v>
       </c>
       <c r="J11" t="n">
-        <v>0.089</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="K11" t="n">
-        <v>0.127</v>
+        <v>0.103</v>
       </c>
       <c r="L11" t="n">
-        <v>0.279</v>
+        <v>0.378</v>
       </c>
       <c r="M11" t="n">
-        <v>0.11</v>
+        <v>0.137</v>
       </c>
       <c r="N11" t="n">
-        <v>0.186</v>
+        <v>0.196</v>
       </c>
       <c r="O11" t="n">
-        <v>0.471</v>
+        <v>0.447</v>
       </c>
       <c r="P11" t="n">
-        <v>2.023</v>
+        <v>1.447</v>
       </c>
       <c r="Q11" t="n">
-        <v>2.513</v>
+        <v>2.537</v>
       </c>
       <c r="R11" t="n">
-        <v>0.353</v>
+        <v>0.26</v>
       </c>
       <c r="S11" t="n">
-        <v>0.482</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="T11" t="n">
         <v>0</v>
       </c>
       <c r="U11" t="n">
-        <v>0.023</v>
+        <v>0.034</v>
       </c>
       <c r="V11" t="n">
-        <v>0.017</v>
+        <v>0.038</v>
       </c>
       <c r="W11" t="n">
-        <v>0.065</v>
+        <v>0.081</v>
       </c>
       <c r="X11" t="n">
-        <v>0.056</v>
+        <v>0.077</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.107</v>
+        <v>0.127</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.079</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="AA11" t="n">
         <v>0.117</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.077</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.109</v>
+        <v>0.097</v>
       </c>
       <c r="AD11" t="n">
-        <v>0.062</v>
+        <v>0.052</v>
       </c>
       <c r="AE11" t="n">
-        <v>0.079</v>
+        <v>0.057</v>
       </c>
       <c r="AF11" t="n">
-        <v>0.042</v>
+        <v>0.035</v>
       </c>
       <c r="AG11" t="n">
-        <v>0.05</v>
+        <v>0.041</v>
       </c>
       <c r="AH11" t="n">
-        <v>0.027</v>
+        <v>0.026</v>
       </c>
       <c r="AI11" t="n">
-        <v>0.024</v>
+        <v>0.016</v>
       </c>
       <c r="AJ11" t="n">
-        <v>0.017</v>
+        <v>0.012</v>
       </c>
       <c r="AK11" t="n">
-        <v>0.014</v>
+        <v>0.011</v>
       </c>
       <c r="AL11" t="n">
-        <v>0.007</v>
+        <v>0.004</v>
       </c>
       <c r="AM11" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="AN11" t="n">
         <v>0.008</v>
-      </c>
-      <c r="AN11" t="n">
-        <v>0.01</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>823479</v>
+        <v>823642</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1909,126 +1909,126 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ARI</t>
+          <t>ATH</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>PHI</t>
+          <t>NYM</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>4.257</v>
+        <v>3.23</v>
       </c>
       <c r="F12" t="n">
-        <v>4.543</v>
+        <v>3.59</v>
       </c>
       <c r="G12" t="n">
-        <v>0.436</v>
+        <v>0.426</v>
       </c>
       <c r="H12" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.574</v>
       </c>
       <c r="I12" t="n">
-        <v>0.25</v>
+        <v>0.184</v>
       </c>
       <c r="J12" t="n">
-        <v>0.079</v>
+        <v>0.107</v>
       </c>
       <c r="K12" t="n">
-        <v>0.106</v>
+        <v>0.135</v>
       </c>
       <c r="L12" t="n">
-        <v>0.267</v>
+        <v>0.245</v>
       </c>
       <c r="M12" t="n">
-        <v>0.113</v>
+        <v>0.121</v>
       </c>
       <c r="N12" t="n">
-        <v>0.184</v>
+        <v>0.207</v>
       </c>
       <c r="O12" t="n">
-        <v>0.481</v>
+        <v>0.404</v>
       </c>
       <c r="P12" t="n">
-        <v>2.339</v>
+        <v>1.647</v>
       </c>
       <c r="Q12" t="n">
-        <v>2.536</v>
+        <v>1.977</v>
       </c>
       <c r="R12" t="n">
-        <v>0.401</v>
+        <v>0.354</v>
       </c>
       <c r="S12" t="n">
-        <v>0.452</v>
+        <v>0.451</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
       </c>
       <c r="U12" t="n">
-        <v>0.015</v>
+        <v>0.042</v>
       </c>
       <c r="V12" t="n">
-        <v>0.019</v>
+        <v>0.043</v>
       </c>
       <c r="W12" t="n">
-        <v>0.064</v>
+        <v>0.11</v>
       </c>
       <c r="X12" t="n">
-        <v>0.053</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.1</v>
+        <v>0.139</v>
       </c>
       <c r="Z12" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>0.123</v>
+      </c>
+      <c r="AB12" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="AA12" t="n">
-        <v>0.109</v>
-      </c>
-      <c r="AB12" t="n">
-        <v>0.08</v>
-      </c>
       <c r="AC12" t="n">
-        <v>0.105</v>
+        <v>0.081</v>
       </c>
       <c r="AD12" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.054</v>
       </c>
       <c r="AE12" t="n">
-        <v>0.075</v>
+        <v>0.055</v>
       </c>
       <c r="AF12" t="n">
-        <v>0.053</v>
+        <v>0.027</v>
       </c>
       <c r="AG12" t="n">
-        <v>0.049</v>
+        <v>0.027</v>
       </c>
       <c r="AH12" t="n">
-        <v>0.031</v>
+        <v>0.014</v>
       </c>
       <c r="AI12" t="n">
-        <v>0.031</v>
+        <v>0.014</v>
       </c>
       <c r="AJ12" t="n">
-        <v>0.021</v>
+        <v>0.006</v>
       </c>
       <c r="AK12" t="n">
-        <v>0.018</v>
+        <v>0.002</v>
       </c>
       <c r="AL12" t="n">
-        <v>0.01</v>
+        <v>0.003</v>
       </c>
       <c r="AM12" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="AN12" t="n">
         <v>0.006</v>
-      </c>
-      <c r="AN12" t="n">
-        <v>0.019</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>823804</v>
+        <v>824126</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -2037,126 +2037,126 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>WAS</t>
+          <t>CHW</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MIL</t>
+          <t xml:space="preserve">KC </t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>3.665</v>
+        <v>4.254</v>
       </c>
       <c r="F13" t="n">
-        <v>4.711</v>
+        <v>5.326</v>
       </c>
       <c r="G13" t="n">
-        <v>0.353</v>
+        <v>0.373</v>
       </c>
       <c r="H13" t="n">
-        <v>0.647</v>
+        <v>0.627</v>
       </c>
       <c r="I13" t="n">
-        <v>0.187</v>
+        <v>0.174</v>
       </c>
       <c r="J13" t="n">
-        <v>0.065</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="K13" t="n">
-        <v>0.101</v>
+        <v>0.113</v>
       </c>
       <c r="L13" t="n">
-        <v>0.339</v>
+        <v>0.338</v>
       </c>
       <c r="M13" t="n">
-        <v>0.12</v>
+        <v>0.107</v>
       </c>
       <c r="N13" t="n">
-        <v>0.189</v>
+        <v>0.182</v>
       </c>
       <c r="O13" t="n">
-        <v>0.468</v>
+        <v>0.495</v>
       </c>
       <c r="P13" t="n">
-        <v>1.918</v>
+        <v>2.404</v>
       </c>
       <c r="Q13" t="n">
-        <v>2.551</v>
+        <v>3.025</v>
       </c>
       <c r="R13" t="n">
-        <v>0.333</v>
+        <v>0.366</v>
       </c>
       <c r="S13" t="n">
-        <v>0.496</v>
+        <v>0.491</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
       </c>
       <c r="U13" t="n">
-        <v>0.016</v>
+        <v>0.011</v>
       </c>
       <c r="V13" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="W13" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="X13" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>0.077</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>0.062</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>0.116</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>0.078</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>0.114</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>0.063</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="AK13" t="n">
         <v>0.024</v>
       </c>
-      <c r="W13" t="n">
-        <v>0.063</v>
-      </c>
-      <c r="X13" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="Y13" t="n">
-        <v>0.107</v>
-      </c>
-      <c r="Z13" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AA13" t="n">
-        <v>0.129</v>
-      </c>
-      <c r="AB13" t="n">
-        <v>0.08400000000000001</v>
-      </c>
-      <c r="AC13" t="n">
-        <v>0.106</v>
-      </c>
-      <c r="AD13" t="n">
-        <v>0.067</v>
-      </c>
-      <c r="AE13" t="n">
-        <v>0.077</v>
-      </c>
-      <c r="AF13" t="n">
-        <v>0.043</v>
-      </c>
-      <c r="AG13" t="n">
-        <v>0.049</v>
-      </c>
-      <c r="AH13" t="n">
-        <v>0.022</v>
-      </c>
-      <c r="AI13" t="n">
-        <v>0.026</v>
-      </c>
-      <c r="AJ13" t="n">
+      <c r="AL13" t="n">
         <v>0.013</v>
       </c>
-      <c r="AK13" t="n">
-        <v>0.014</v>
-      </c>
-      <c r="AL13" t="n">
-        <v>0.005</v>
-      </c>
       <c r="AM13" t="n">
-        <v>0.007</v>
+        <v>0.013</v>
       </c>
       <c r="AN13" t="n">
-        <v>0.015</v>
+        <v>0.024</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>823966</v>
+        <v>824293</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -2165,126 +2165,126 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>TEX</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>4.783</v>
+        <v>3.227</v>
       </c>
       <c r="F14" t="n">
-        <v>3.687</v>
+        <v>3.586</v>
       </c>
       <c r="G14" t="n">
-        <v>0.579</v>
+        <v>0.433</v>
       </c>
       <c r="H14" t="n">
-        <v>0.421</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="I14" t="n">
-        <v>0.33</v>
+        <v>0.194</v>
       </c>
       <c r="J14" t="n">
-        <v>0.118</v>
+        <v>0.1</v>
       </c>
       <c r="K14" t="n">
-        <v>0.131</v>
+        <v>0.14</v>
       </c>
       <c r="L14" t="n">
-        <v>0.158</v>
+        <v>0.239</v>
       </c>
       <c r="M14" t="n">
-        <v>0.081</v>
+        <v>0.125</v>
       </c>
       <c r="N14" t="n">
-        <v>0.182</v>
+        <v>0.203</v>
       </c>
       <c r="O14" t="n">
-        <v>0.498</v>
+        <v>0.388</v>
       </c>
       <c r="P14" t="n">
-        <v>2.799</v>
+        <v>1.524</v>
       </c>
       <c r="Q14" t="n">
-        <v>1.852</v>
+        <v>1.909</v>
       </c>
       <c r="R14" t="n">
-        <v>0.541</v>
+        <v>0.344</v>
       </c>
       <c r="S14" t="n">
-        <v>0.293</v>
+        <v>0.454</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
       </c>
       <c r="U14" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="V14" t="n">
+        <v>0.039</v>
+      </c>
+      <c r="W14" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>0.126</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>0.124</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>0.081</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>0.082</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>0.047</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="AH14" t="n">
         <v>0.016</v>
       </c>
-      <c r="V14" t="n">
-        <v>0.019</v>
-      </c>
-      <c r="W14" t="n">
-        <v>0.067</v>
-      </c>
-      <c r="X14" t="n">
-        <v>0.055</v>
-      </c>
-      <c r="Y14" t="n">
-        <v>0.102</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="AA14" t="n">
-        <v>0.127</v>
-      </c>
-      <c r="AB14" t="n">
-        <v>0.077</v>
-      </c>
-      <c r="AC14" t="n">
-        <v>0.109</v>
-      </c>
-      <c r="AD14" t="n">
-        <v>0.061</v>
-      </c>
-      <c r="AE14" t="n">
-        <v>0.07099999999999999</v>
-      </c>
-      <c r="AF14" t="n">
-        <v>0.048</v>
-      </c>
-      <c r="AG14" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="AH14" t="n">
-        <v>0.03</v>
-      </c>
       <c r="AI14" t="n">
-        <v>0.03</v>
+        <v>0.011</v>
       </c>
       <c r="AJ14" t="n">
-        <v>0.015</v>
+        <v>0.011</v>
       </c>
       <c r="AK14" t="n">
-        <v>0.013</v>
+        <v>0.006</v>
       </c>
       <c r="AL14" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.003</v>
       </c>
       <c r="AM14" t="n">
-        <v>0.005</v>
+        <v>0.003</v>
       </c>
       <c r="AN14" t="n">
-        <v>0.012</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>824533</v>
+        <v>824696</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -2293,126 +2293,126 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>LAA</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CIN</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>3.95</v>
+        <v>5.675</v>
       </c>
       <c r="F15" t="n">
-        <v>4.212</v>
+        <v>5.776</v>
       </c>
       <c r="G15" t="n">
-        <v>0.456</v>
+        <v>0.484</v>
       </c>
       <c r="H15" t="n">
-        <v>0.544</v>
+        <v>0.516</v>
       </c>
       <c r="I15" t="n">
-        <v>0.22</v>
+        <v>0.277</v>
       </c>
       <c r="J15" t="n">
-        <v>0.098</v>
+        <v>0.095</v>
       </c>
       <c r="K15" t="n">
-        <v>0.138</v>
+        <v>0.112</v>
       </c>
       <c r="L15" t="n">
-        <v>0.242</v>
+        <v>0.277</v>
       </c>
       <c r="M15" t="n">
-        <v>0.099</v>
+        <v>0.093</v>
       </c>
       <c r="N15" t="n">
-        <v>0.203</v>
+        <v>0.147</v>
       </c>
       <c r="O15" t="n">
-        <v>0.447</v>
+        <v>0.541</v>
       </c>
       <c r="P15" t="n">
-        <v>2.002</v>
+        <v>2.948</v>
       </c>
       <c r="Q15" t="n">
-        <v>2.257</v>
+        <v>3.095</v>
       </c>
       <c r="R15" t="n">
-        <v>0.385</v>
+        <v>0.439</v>
       </c>
       <c r="S15" t="n">
-        <v>0.445</v>
+        <v>0.433</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
       </c>
       <c r="U15" t="n">
-        <v>0.019</v>
+        <v>0.005</v>
       </c>
       <c r="V15" t="n">
-        <v>0.028</v>
+        <v>0.005</v>
       </c>
       <c r="W15" t="n">
-        <v>0.078</v>
+        <v>0.016</v>
       </c>
       <c r="X15" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>0.082</v>
+      </c>
+      <c r="AB15" t="n">
         <v>0.062</v>
       </c>
-      <c r="Y15" t="n">
-        <v>0.119</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>0.075</v>
-      </c>
-      <c r="AA15" t="n">
-        <v>0.127</v>
-      </c>
-      <c r="AB15" t="n">
-        <v>0.064</v>
-      </c>
       <c r="AC15" t="n">
-        <v>0.105</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="AD15" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>0.08799999999999999</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="AH15" t="n">
+        <v>0.051</v>
+      </c>
+      <c r="AI15" t="n">
         <v>0.063</v>
       </c>
-      <c r="AE15" t="n">
-        <v>0.067</v>
-      </c>
-      <c r="AF15" t="n">
-        <v>0.037</v>
-      </c>
-      <c r="AG15" t="n">
-        <v>0.043</v>
-      </c>
-      <c r="AH15" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="AI15" t="n">
-        <v>0.028</v>
-      </c>
       <c r="AJ15" t="n">
-        <v>0.018</v>
+        <v>0.041</v>
       </c>
       <c r="AK15" t="n">
-        <v>0.02</v>
+        <v>0.042</v>
       </c>
       <c r="AL15" t="n">
-        <v>0.008</v>
+        <v>0.024</v>
       </c>
       <c r="AM15" t="n">
-        <v>0.005</v>
+        <v>0.026</v>
       </c>
       <c r="AN15" t="n">
-        <v>0.01</v>
+        <v>0.065</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>824859</v>
+        <v>824938</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -2421,121 +2421,121 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">SF </t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>BAL</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>4.294</v>
+        <v>3.666</v>
       </c>
       <c r="F16" t="n">
-        <v>4.276</v>
+        <v>4.101</v>
       </c>
       <c r="G16" t="n">
-        <v>0.481</v>
+        <v>0.43</v>
       </c>
       <c r="H16" t="n">
-        <v>0.519</v>
+        <v>0.57</v>
       </c>
       <c r="I16" t="n">
-        <v>0.255</v>
+        <v>0.21</v>
       </c>
       <c r="J16" t="n">
-        <v>0.097</v>
+        <v>0.095</v>
       </c>
       <c r="K16" t="n">
-        <v>0.129</v>
+        <v>0.125</v>
       </c>
       <c r="L16" t="n">
-        <v>0.245</v>
+        <v>0.273</v>
       </c>
       <c r="M16" t="n">
-        <v>0.1</v>
+        <v>0.113</v>
       </c>
       <c r="N16" t="n">
-        <v>0.174</v>
+        <v>0.184</v>
       </c>
       <c r="O16" t="n">
-        <v>0.494</v>
+        <v>0.461</v>
       </c>
       <c r="P16" t="n">
-        <v>2.449</v>
+        <v>1.968</v>
       </c>
       <c r="Q16" t="n">
-        <v>2.38</v>
+        <v>2.361</v>
       </c>
       <c r="R16" t="n">
-        <v>0.434</v>
+        <v>0.363</v>
       </c>
       <c r="S16" t="n">
-        <v>0.411</v>
+        <v>0.475</v>
       </c>
       <c r="T16" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="U16" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="V16" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="W16" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="X16" t="n">
+        <v>0.066</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>0.108</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>0.08799999999999999</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>0.137</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>0.067</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="AH16" t="n">
         <v>0.018</v>
       </c>
-      <c r="V16" t="n">
-        <v>0.021</v>
-      </c>
-      <c r="W16" t="n">
-        <v>0.061</v>
-      </c>
-      <c r="X16" t="n">
-        <v>0.052</v>
-      </c>
-      <c r="Y16" t="n">
-        <v>0.104</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>0.077</v>
-      </c>
-      <c r="AA16" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="AB16" t="n">
-        <v>0.08500000000000001</v>
-      </c>
-      <c r="AC16" t="n">
-        <v>0.099</v>
-      </c>
-      <c r="AD16" t="n">
-        <v>0.064</v>
-      </c>
-      <c r="AE16" t="n">
-        <v>0.079</v>
-      </c>
-      <c r="AF16" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="AG16" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="AH16" t="n">
-        <v>0.031</v>
-      </c>
       <c r="AI16" t="n">
-        <v>0.036</v>
+        <v>0.019</v>
       </c>
       <c r="AJ16" t="n">
         <v>0.015</v>
       </c>
       <c r="AK16" t="n">
-        <v>0.013</v>
+        <v>0.011</v>
       </c>
       <c r="AL16" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.006</v>
       </c>
       <c r="AM16" t="n">
-        <v>0.011</v>
+        <v>0.005</v>
       </c>
       <c r="AN16" t="n">
-        <v>0.012</v>
+        <v>0.005</v>
       </c>
     </row>
   </sheetData>

</xml_diff>